<commit_message>
BOM: H-version Picos (pre-soldered headers); host debug JST replaced by 1x3 header
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/dock/BOM.xlsx
+++ b/hardware/dock/BOM.xlsx
@@ -134,13 +134,13 @@
     <t xml:space="preserve">Host + BLE module</t>
   </si>
   <si>
-    <t xml:space="preserve">Raspberry Pi Pico 2 W</t>
+    <t xml:space="preserve">Raspberry Pi Pico 2 WH</t>
   </si>
   <si>
     <t xml:space="preserve">Socketed, 2×20 headers</t>
   </si>
   <si>
-    <t xml:space="preserve">Solder male 1×20 headers + a 1×3 header on the debug holes (pointing down)</t>
+    <t xml:space="preserve">H version (headers pre-soldered). Remove the JST-SH debug connector and fit a 1×3 male header in the debug holes, pointing down</t>
   </si>
   <si>
     <t xml:space="preserve">A2, A3</t>
@@ -149,10 +149,10 @@
     <t xml:space="preserve">HID endpoint modules</t>
   </si>
   <si>
-    <t xml:space="preserve">Raspberry Pi Pico 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solder male 1×20 headers (pointing down)</t>
+    <t xml:space="preserve">Raspberry Pi Pico 2 H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H version (headers pre-soldered). JST debug connector can stay; SWD is via pogo probes on the bottom pads</t>
   </si>
   <si>
     <t xml:space="preserve">ICs</t>
@@ -416,19 +416,19 @@
     <t xml:space="preserve">Female socket 1×3, 2.54 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">Host SWD (under the Pico 2 W debug holes); can be cut from a longer strip</t>
+    <t xml:space="preserve">On the dock, under the host Pico 2 WH debug holes</t>
   </si>
   <si>
     <t xml:space="preserve">Male pin header 1×20, 2.54 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">Soldered to the Picos</t>
+    <t xml:space="preserve">Not needed: H-version Picos come with headers pre-soldered</t>
   </si>
   <si>
     <t xml:space="preserve">Male pin header 1×3, 2.54 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">Host debug holes</t>
+    <t xml:space="preserve">Replaces the JST-SH debug connector on the host Pico 2 WH, pointing down into the 1×3 socket</t>
   </si>
   <si>
     <t xml:space="preserve">Spring probe P50-B1</t>
@@ -629,32 +629,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -706,7 +710,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1068,1473 +1072,1473 @@
   <dimension ref="A1:P38"/>
   <sheetFormatPr defaultColWidth="8.6171875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="46"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="3" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="6" t="n">
         <f aca="false">SUM(M10:M37)</f>
         <v>459.81</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="4" t="n">
         <f aca="false">COUNT(L10:L37)</f>
         <v>5</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="4" t="n">
         <f aca="false">COUNTBLANK(L10:L37)</f>
         <v>23</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="7" t="s">
+      <c r="J9" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="7" t="s">
+      <c r="K9" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="L9" s="7" t="s">
+      <c r="L9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="M9" s="7" t="s">
+      <c r="M9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="N9" s="7" t="s">
+      <c r="N9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="O9" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="P9" s="7" t="s">
+      <c r="P9" s="8" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="9" t="s">
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="12" t="n">
+      <c r="G10" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="I10" s="9" t="n">
         <f aca="false">G10*$C$4+H10</f>
         <v>1</v>
       </c>
-      <c r="J10" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="8" t="n">
+      <c r="J10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="9" t="n">
         <f aca="false">IF(I10&lt;=0,0,ROUNDUP(I10/J10,0))</f>
         <v>1</v>
       </c>
-      <c r="L10" s="13"/>
-      <c r="M10" s="14" t="str">
+      <c r="L10" s="14"/>
+      <c r="M10" s="15" t="str">
         <f aca="false">IF(L10="","",K10*L10)</f>
         <v/>
       </c>
-      <c r="N10" s="15"/>
-      <c r="O10" s="15"/>
-      <c r="P10" s="16" t="s">
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
+      <c r="P10" s="17" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" s="8" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" s="12" t="n">
+      <c r="G11" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I11" s="9" t="n">
         <f aca="false">G11*$C$4+H11</f>
         <v>2</v>
       </c>
-      <c r="J11" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" s="8" t="n">
+      <c r="J11" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="9" t="n">
         <f aca="false">IF(I11&lt;=0,0,ROUNDUP(I11/J11,0))</f>
         <v>2</v>
       </c>
-      <c r="L11" s="13"/>
-      <c r="M11" s="14" t="str">
+      <c r="L11" s="14"/>
+      <c r="M11" s="15" t="str">
         <f aca="false">IF(L11="","",K11*L11)</f>
         <v/>
       </c>
-      <c r="N11" s="15"/>
-      <c r="O11" s="15"/>
-      <c r="P11" s="16" t="s">
+      <c r="N11" s="16"/>
+      <c r="O11" s="16"/>
+      <c r="P11" s="17" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I12" s="8" t="n">
+      <c r="G12" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" s="9" t="n">
         <f aca="false">G12*$C$4+H12</f>
         <v>3</v>
       </c>
-      <c r="J12" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="8" t="n">
+      <c r="J12" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="9" t="n">
         <f aca="false">IF(I12&lt;=0,0,ROUNDUP(I12/J12,0))</f>
         <v>3</v>
       </c>
-      <c r="L12" s="13"/>
-      <c r="M12" s="14" t="str">
+      <c r="L12" s="14"/>
+      <c r="M12" s="15" t="str">
         <f aca="false">IF(L12="","",K12*L12)</f>
         <v/>
       </c>
-      <c r="N12" s="15" t="s">
+      <c r="N12" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="O12" s="17" t="s">
+      <c r="O12" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="P12" s="16" t="s">
+      <c r="P12" s="17" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="G13" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="8" t="n">
+      <c r="G13" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="9" t="n">
         <f aca="false">G13*$C$4+H13</f>
         <v>2</v>
       </c>
-      <c r="J13" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="8" t="n">
+      <c r="J13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="9" t="n">
         <f aca="false">IF(I13&lt;=0,0,ROUNDUP(I13/J13,0))</f>
         <v>2</v>
       </c>
-      <c r="L13" s="18" t="n">
+      <c r="L13" s="19" t="n">
         <v>26.81</v>
       </c>
-      <c r="M13" s="14" t="n">
+      <c r="M13" s="15" t="n">
         <f aca="false">IF(L13="","",K13*L13)</f>
         <v>53.62</v>
       </c>
-      <c r="N13" s="15" t="s">
+      <c r="N13" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="O13" s="17" t="s">
+      <c r="O13" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="P13" s="16" t="s">
+      <c r="P13" s="17" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="G14" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" s="8" t="n">
+      <c r="G14" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="9" t="n">
         <f aca="false">G14*$C$4+H14</f>
         <v>2</v>
       </c>
-      <c r="J14" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" s="8" t="n">
+      <c r="J14" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="9" t="n">
         <f aca="false">IF(I14&lt;=0,0,ROUNDUP(I14/J14,0))</f>
         <v>2</v>
       </c>
-      <c r="L14" s="18" t="n">
+      <c r="L14" s="19" t="n">
         <v>27.02</v>
       </c>
-      <c r="M14" s="14" t="n">
+      <c r="M14" s="15" t="n">
         <f aca="false">IF(L14="","",K14*L14)</f>
         <v>54.04</v>
       </c>
-      <c r="N14" s="15" t="s">
+      <c r="N14" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="O14" s="17" t="s">
+      <c r="O14" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="P14" s="16" t="s">
+      <c r="P14" s="17" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G15" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H15" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I15" s="8" t="n">
+      <c r="H15" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I15" s="9" t="n">
         <f aca="false">G15*$C$4+H15</f>
         <v>6</v>
       </c>
-      <c r="J15" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="8" t="n">
+      <c r="J15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="9" t="n">
         <f aca="false">IF(I15&lt;=0,0,ROUNDUP(I15/J15,0))</f>
         <v>6</v>
       </c>
-      <c r="L15" s="18" t="n">
+      <c r="L15" s="19" t="n">
         <v>11.88</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="M15" s="15" t="n">
         <f aca="false">IF(L15="","",K15*L15)</f>
         <v>71.28</v>
       </c>
-      <c r="N15" s="15" t="s">
+      <c r="N15" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="O15" s="17" t="s">
+      <c r="O15" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="P15" s="16" t="s">
+      <c r="P15" s="17" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F16" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G16" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H16" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I16" s="8" t="n">
+      <c r="H16" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" s="9" t="n">
         <f aca="false">G16*$C$4+H16</f>
         <v>5</v>
       </c>
-      <c r="J16" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" s="8" t="n">
+      <c r="J16" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="9" t="n">
         <f aca="false">IF(I16&lt;=0,0,ROUNDUP(I16/J16,0))</f>
         <v>5</v>
       </c>
-      <c r="L16" s="13"/>
-      <c r="M16" s="14" t="str">
+      <c r="L16" s="14"/>
+      <c r="M16" s="15" t="str">
         <f aca="false">IF(L16="","",K16*L16)</f>
         <v/>
       </c>
-      <c r="N16" s="15"/>
-      <c r="O16" s="15"/>
-      <c r="P16" s="16" t="s">
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="17" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="n">
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F17" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="12" t="n">
+      <c r="G17" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="8" t="n">
+      <c r="I17" s="9" t="n">
         <f aca="false">G17*$C$4+H17</f>
         <v>1</v>
       </c>
-      <c r="J17" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="8" t="n">
+      <c r="J17" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="9" t="n">
         <f aca="false">IF(I17&lt;=0,0,ROUNDUP(I17/J17,0))</f>
         <v>1</v>
       </c>
-      <c r="L17" s="13"/>
-      <c r="M17" s="14" t="str">
+      <c r="L17" s="14"/>
+      <c r="M17" s="15" t="str">
         <f aca="false">IF(L17="","",K17*L17)</f>
         <v/>
       </c>
-      <c r="N17" s="15"/>
-      <c r="O17" s="15"/>
-      <c r="P17" s="16" t="s">
+      <c r="N17" s="16"/>
+      <c r="O17" s="16"/>
+      <c r="P17" s="17" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="G18" s="11" t="n">
+      <c r="G18" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H18" s="12" t="n">
+      <c r="H18" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="I18" s="8" t="n">
+      <c r="I18" s="9" t="n">
         <f aca="false">G18*$C$4+H18</f>
         <v>3</v>
       </c>
-      <c r="J18" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" s="8" t="n">
+      <c r="J18" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="9" t="n">
         <f aca="false">IF(I18&lt;=0,0,ROUNDUP(I18/J18,0))</f>
         <v>3</v>
       </c>
-      <c r="L18" s="13"/>
-      <c r="M18" s="14" t="str">
+      <c r="L18" s="14"/>
+      <c r="M18" s="15" t="str">
         <f aca="false">IF(L18="","",K18*L18)</f>
         <v/>
       </c>
-      <c r="N18" s="15"/>
-      <c r="O18" s="15"/>
-      <c r="P18" s="16" t="s">
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="17" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="n">
+    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="F19" s="10" t="s">
+      <c r="F19" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="G19" s="11" t="n">
+      <c r="G19" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H19" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" s="8" t="n">
+      <c r="H19" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="9" t="n">
         <f aca="false">G19*$C$4+H19</f>
         <v>5</v>
       </c>
-      <c r="J19" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" s="8" t="n">
+      <c r="J19" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="9" t="n">
         <f aca="false">IF(I19&lt;=0,0,ROUNDUP(I19/J19,0))</f>
         <v>5</v>
       </c>
-      <c r="L19" s="18" t="n">
+      <c r="L19" s="19" t="n">
         <v>14.33</v>
       </c>
-      <c r="M19" s="14" t="n">
+      <c r="M19" s="15" t="n">
         <f aca="false">IF(L19="","",K19*L19)</f>
         <v>71.65</v>
       </c>
-      <c r="N19" s="15" t="s">
+      <c r="N19" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="O19" s="17" t="s">
+      <c r="O19" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="P19" s="16" t="s">
+      <c r="P19" s="17" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="G20" s="11" t="n">
+      <c r="G20" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="H20" s="12" t="n">
+      <c r="H20" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="I20" s="8" t="n">
+      <c r="I20" s="9" t="n">
         <f aca="false">G20*$C$4+H20</f>
         <v>10</v>
       </c>
-      <c r="J20" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="8" t="n">
+      <c r="J20" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="9" t="n">
         <f aca="false">IF(I20&lt;=0,0,ROUNDUP(I20/J20,0))</f>
         <v>10</v>
       </c>
-      <c r="L20" s="13"/>
-      <c r="M20" s="14" t="str">
+      <c r="L20" s="14"/>
+      <c r="M20" s="15" t="str">
         <f aca="false">IF(L20="","",K20*L20)</f>
         <v/>
       </c>
-      <c r="N20" s="15"/>
-      <c r="O20" s="15"/>
-      <c r="P20" s="16"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="n">
+      <c r="N20" s="16"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="17"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="G21" s="11" t="n">
+      <c r="G21" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H21" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I21" s="8" t="n">
+      <c r="H21" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" s="9" t="n">
         <f aca="false">G21*$C$4+H21</f>
         <v>5</v>
       </c>
-      <c r="J21" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" s="8" t="n">
+      <c r="J21" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="9" t="n">
         <f aca="false">IF(I21&lt;=0,0,ROUNDUP(I21/J21,0))</f>
         <v>5</v>
       </c>
-      <c r="L21" s="13"/>
-      <c r="M21" s="14" t="str">
+      <c r="L21" s="14"/>
+      <c r="M21" s="15" t="str">
         <f aca="false">IF(L21="","",K21*L21)</f>
         <v/>
       </c>
-      <c r="N21" s="15"/>
-      <c r="O21" s="15"/>
-      <c r="P21" s="16" t="s">
+      <c r="N21" s="16"/>
+      <c r="O21" s="16"/>
+      <c r="P21" s="17" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="n">
+    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="F22" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G22" s="11" t="n">
+      <c r="G22" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="H22" s="12" t="n">
+      <c r="H22" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="I22" s="8" t="n">
+      <c r="I22" s="9" t="n">
         <f aca="false">G22*$C$4+H22</f>
         <v>15</v>
       </c>
-      <c r="J22" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K22" s="8" t="n">
+      <c r="J22" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="9" t="n">
         <f aca="false">IF(I22&lt;=0,0,ROUNDUP(I22/J22,0))</f>
         <v>15</v>
       </c>
-      <c r="L22" s="13"/>
-      <c r="M22" s="14" t="str">
+      <c r="L22" s="14"/>
+      <c r="M22" s="15" t="str">
         <f aca="false">IF(L22="","",K22*L22)</f>
         <v/>
       </c>
-      <c r="N22" s="15"/>
-      <c r="O22" s="15"/>
-      <c r="P22" s="16"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="n">
+      <c r="N22" s="16"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="17"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="E23" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F23" s="10" t="s">
+      <c r="F23" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G23" s="11" t="n">
+      <c r="G23" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H23" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I23" s="8" t="n">
+      <c r="H23" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" s="9" t="n">
         <f aca="false">G23*$C$4+H23</f>
         <v>7</v>
       </c>
-      <c r="J23" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K23" s="8" t="n">
+      <c r="J23" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="9" t="n">
         <f aca="false">IF(I23&lt;=0,0,ROUNDUP(I23/J23,0))</f>
         <v>7</v>
       </c>
-      <c r="L23" s="13"/>
-      <c r="M23" s="14" t="str">
+      <c r="L23" s="14"/>
+      <c r="M23" s="15" t="str">
         <f aca="false">IF(L23="","",K23*L23)</f>
         <v/>
       </c>
-      <c r="N23" s="15"/>
-      <c r="O23" s="15"/>
-      <c r="P23" s="16"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="n">
+      <c r="N23" s="16"/>
+      <c r="O23" s="16"/>
+      <c r="P23" s="17"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F24" s="10" t="s">
+      <c r="F24" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G24" s="11" t="n">
+      <c r="G24" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H24" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I24" s="8" t="n">
+      <c r="H24" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I24" s="9" t="n">
         <f aca="false">G24*$C$4+H24</f>
         <v>6</v>
       </c>
-      <c r="J24" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K24" s="8" t="n">
+      <c r="J24" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" s="9" t="n">
         <f aca="false">IF(I24&lt;=0,0,ROUNDUP(I24/J24,0))</f>
         <v>6</v>
       </c>
-      <c r="L24" s="13"/>
-      <c r="M24" s="14" t="str">
+      <c r="L24" s="14"/>
+      <c r="M24" s="15" t="str">
         <f aca="false">IF(L24="","",K24*L24)</f>
         <v/>
       </c>
-      <c r="N24" s="15"/>
-      <c r="O24" s="15"/>
-      <c r="P24" s="16" t="s">
+      <c r="N24" s="16"/>
+      <c r="O24" s="16"/>
+      <c r="P24" s="17" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E25" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F25" s="10" t="s">
+      <c r="F25" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G25" s="11" t="n">
+      <c r="G25" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H25" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I25" s="8" t="n">
+      <c r="H25" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="9" t="n">
         <f aca="false">G25*$C$4+H25</f>
         <v>5</v>
       </c>
-      <c r="J25" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" s="8" t="n">
+      <c r="J25" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" s="9" t="n">
         <f aca="false">IF(I25&lt;=0,0,ROUNDUP(I25/J25,0))</f>
         <v>5</v>
       </c>
-      <c r="L25" s="13"/>
-      <c r="M25" s="14" t="str">
+      <c r="L25" s="14"/>
+      <c r="M25" s="15" t="str">
         <f aca="false">IF(L25="","",K25*L25)</f>
         <v/>
       </c>
-      <c r="N25" s="15"/>
-      <c r="O25" s="15"/>
-      <c r="P25" s="16"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="n">
+      <c r="N25" s="16"/>
+      <c r="O25" s="16"/>
+      <c r="P25" s="17"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="n">
         <v>17</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F26" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G26" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H26" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I26" s="8" t="n">
+      <c r="G26" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" s="9" t="n">
         <f aca="false">G26*$C$4+H26</f>
         <v>4</v>
       </c>
-      <c r="J26" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K26" s="8" t="n">
+      <c r="J26" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" s="9" t="n">
         <f aca="false">IF(I26&lt;=0,0,ROUNDUP(I26/J26,0))</f>
         <v>4</v>
       </c>
-      <c r="L26" s="13"/>
-      <c r="M26" s="14" t="str">
+      <c r="L26" s="14"/>
+      <c r="M26" s="15" t="str">
         <f aca="false">IF(L26="","",K26*L26)</f>
         <v/>
       </c>
-      <c r="N26" s="15"/>
-      <c r="O26" s="15"/>
-      <c r="P26" s="16" t="s">
+      <c r="N26" s="16"/>
+      <c r="O26" s="16"/>
+      <c r="P26" s="17" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="E27" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="F27" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G27" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H27" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I27" s="8" t="n">
+      <c r="G27" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I27" s="9" t="n">
         <f aca="false">G27*$C$4+H27</f>
         <v>4</v>
       </c>
-      <c r="J27" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K27" s="8" t="n">
+      <c r="J27" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" s="9" t="n">
         <f aca="false">IF(I27&lt;=0,0,ROUNDUP(I27/J27,0))</f>
         <v>4</v>
       </c>
-      <c r="L27" s="13"/>
-      <c r="M27" s="14" t="str">
+      <c r="L27" s="14"/>
+      <c r="M27" s="15" t="str">
         <f aca="false">IF(L27="","",K27*L27)</f>
         <v/>
       </c>
-      <c r="N27" s="15"/>
-      <c r="O27" s="15"/>
-      <c r="P27" s="16" t="s">
+      <c r="N27" s="16"/>
+      <c r="O27" s="16"/>
+      <c r="P27" s="17" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="n">
         <v>19</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="E28" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F28" s="10" t="s">
+      <c r="F28" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H28" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I28" s="8" t="n">
+      <c r="G28" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I28" s="9" t="n">
         <f aca="false">G28*$C$4+H28</f>
         <v>4</v>
       </c>
-      <c r="J28" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K28" s="8" t="n">
+      <c r="J28" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" s="9" t="n">
         <f aca="false">IF(I28&lt;=0,0,ROUNDUP(I28/J28,0))</f>
         <v>4</v>
       </c>
-      <c r="L28" s="13"/>
-      <c r="M28" s="14" t="str">
+      <c r="L28" s="14"/>
+      <c r="M28" s="15" t="str">
         <f aca="false">IF(L28="","",K28*L28)</f>
         <v/>
       </c>
-      <c r="N28" s="15"/>
-      <c r="O28" s="15"/>
-      <c r="P28" s="16" t="s">
+      <c r="N28" s="16"/>
+      <c r="O28" s="16"/>
+      <c r="P28" s="17" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="E29" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F29" s="10" t="s">
+      <c r="F29" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G29" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H29" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I29" s="8" t="n">
+      <c r="G29" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I29" s="9" t="n">
         <f aca="false">G29*$C$4+H29</f>
         <v>4</v>
       </c>
-      <c r="J29" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K29" s="8" t="n">
+      <c r="J29" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="9" t="n">
         <f aca="false">IF(I29&lt;=0,0,ROUNDUP(I29/J29,0))</f>
         <v>4</v>
       </c>
-      <c r="L29" s="13"/>
-      <c r="M29" s="14" t="str">
+      <c r="L29" s="14"/>
+      <c r="M29" s="15" t="str">
         <f aca="false">IF(L29="","",K29*L29)</f>
         <v/>
       </c>
-      <c r="N29" s="15"/>
-      <c r="O29" s="15"/>
-      <c r="P29" s="16" t="s">
+      <c r="N29" s="16"/>
+      <c r="O29" s="16"/>
+      <c r="P29" s="17" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="E30" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F30" s="10" t="s">
+      <c r="F30" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G30" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H30" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I30" s="8" t="n">
+      <c r="G30" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I30" s="9" t="n">
         <f aca="false">G30*$C$4+H30</f>
         <v>4</v>
       </c>
-      <c r="J30" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K30" s="8" t="n">
+      <c r="J30" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" s="9" t="n">
         <f aca="false">IF(I30&lt;=0,0,ROUNDUP(I30/J30,0))</f>
         <v>4</v>
       </c>
-      <c r="L30" s="13"/>
-      <c r="M30" s="14" t="str">
+      <c r="L30" s="14"/>
+      <c r="M30" s="15" t="str">
         <f aca="false">IF(L30="","",K30*L30)</f>
         <v/>
       </c>
-      <c r="N30" s="15"/>
-      <c r="O30" s="15"/>
-      <c r="P30" s="16"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="8" t="n">
+      <c r="N30" s="16"/>
+      <c r="O30" s="16"/>
+      <c r="P30" s="17"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="D31" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="E31" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F31" s="10" t="s">
+      <c r="F31" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G31" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H31" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I31" s="8" t="n">
+      <c r="G31" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I31" s="9" t="n">
         <f aca="false">G31*$C$4+H31</f>
         <v>3</v>
       </c>
-      <c r="J31" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K31" s="8" t="n">
+      <c r="J31" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K31" s="9" t="n">
         <f aca="false">IF(I31&lt;=0,0,ROUNDUP(I31/J31,0))</f>
         <v>3</v>
       </c>
-      <c r="L31" s="13"/>
-      <c r="M31" s="14" t="str">
+      <c r="L31" s="14"/>
+      <c r="M31" s="15" t="str">
         <f aca="false">IF(L31="","",K31*L31)</f>
         <v/>
       </c>
-      <c r="N31" s="15"/>
-      <c r="O31" s="15"/>
-      <c r="P31" s="16" t="s">
+      <c r="N31" s="16"/>
+      <c r="O31" s="16"/>
+      <c r="P31" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="8" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B32" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="E32" s="10" t="s">
+      <c r="E32" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F32" s="10" t="s">
+      <c r="F32" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="G32" s="11" t="n">
+      <c r="G32" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H32" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I32" s="8" t="n">
+      <c r="H32" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="9" t="n">
         <f aca="false">G32*$C$4+H32</f>
         <v>7</v>
       </c>
-      <c r="J32" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K32" s="8" t="n">
+      <c r="J32" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" s="9" t="n">
         <f aca="false">IF(I32&lt;=0,0,ROUNDUP(I32/J32,0))</f>
         <v>7</v>
       </c>
-      <c r="L32" s="13"/>
-      <c r="M32" s="14" t="str">
+      <c r="L32" s="14"/>
+      <c r="M32" s="15" t="str">
         <f aca="false">IF(L32="","",K32*L32)</f>
         <v/>
       </c>
-      <c r="N32" s="15"/>
-      <c r="O32" s="15"/>
-      <c r="P32" s="16" t="s">
+      <c r="N32" s="16"/>
+      <c r="O32" s="16"/>
+      <c r="P32" s="17" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="n">
+    <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D33" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="E33" s="10" t="s">
+      <c r="E33" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="10" t="s">
+      <c r="F33" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="G33" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H33" s="12" t="n">
+      <c r="G33" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="I33" s="8" t="n">
+      <c r="I33" s="9" t="n">
         <f aca="false">G33*$C$4+H33</f>
         <v>1</v>
       </c>
-      <c r="J33" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K33" s="8" t="n">
+      <c r="J33" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="9" t="n">
         <f aca="false">IF(I33&lt;=0,0,ROUNDUP(I33/J33,0))</f>
         <v>1</v>
       </c>
-      <c r="L33" s="13"/>
-      <c r="M33" s="14" t="str">
+      <c r="L33" s="14"/>
+      <c r="M33" s="15" t="str">
         <f aca="false">IF(L33="","",K33*L33)</f>
         <v/>
       </c>
-      <c r="N33" s="15"/>
-      <c r="O33" s="15"/>
-      <c r="P33" s="16" t="s">
+      <c r="N33" s="16"/>
+      <c r="O33" s="16"/>
+      <c r="P33" s="17" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="8" t="n">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C34" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="D34" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="E34" s="10" t="s">
+      <c r="E34" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F34" s="10" t="s">
+      <c r="F34" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="G34" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="H34" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I34" s="8" t="n">
+      <c r="G34" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="9" t="n">
         <f aca="false">G34*$C$4+H34</f>
-        <v>7</v>
-      </c>
-      <c r="J34" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" s="9" t="n">
         <f aca="false">IF(I34&lt;=0,0,ROUNDUP(I34/J34,0))</f>
-        <v>7</v>
-      </c>
-      <c r="L34" s="13"/>
-      <c r="M34" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="L34" s="14"/>
+      <c r="M34" s="15" t="str">
         <f aca="false">IF(L34="","",K34*L34)</f>
         <v/>
       </c>
-      <c r="N34" s="15"/>
-      <c r="O34" s="15"/>
-      <c r="P34" s="16" t="s">
+      <c r="N34" s="16"/>
+      <c r="O34" s="16"/>
+      <c r="P34" s="17" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="8" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="C35" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="E35" s="10" t="s">
+      <c r="E35" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F35" s="10" t="s">
+      <c r="F35" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="G35" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H35" s="12" t="n">
+      <c r="G35" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="I35" s="8" t="n">
+      <c r="I35" s="9" t="n">
         <f aca="false">G35*$C$4+H35</f>
         <v>1</v>
       </c>
-      <c r="J35" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K35" s="8" t="n">
+      <c r="J35" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" s="9" t="n">
         <f aca="false">IF(I35&lt;=0,0,ROUNDUP(I35/J35,0))</f>
         <v>1</v>
       </c>
-      <c r="L35" s="13"/>
-      <c r="M35" s="14" t="str">
+      <c r="L35" s="14"/>
+      <c r="M35" s="15" t="str">
         <f aca="false">IF(L35="","",K35*L35)</f>
         <v/>
       </c>
-      <c r="N35" s="15"/>
-      <c r="O35" s="15"/>
-      <c r="P35" s="16" t="s">
+      <c r="N35" s="16"/>
+      <c r="O35" s="16"/>
+      <c r="P35" s="17" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="8" t="n">
+    <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="C36" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D36" s="10" t="s">
+      <c r="D36" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="E36" s="10" t="s">
+      <c r="E36" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="F36" s="10" t="s">
+      <c r="F36" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="G36" s="11" t="n">
+      <c r="G36" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="H36" s="12" t="n">
+      <c r="H36" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="I36" s="8" t="n">
+      <c r="I36" s="9" t="n">
         <f aca="false">G36*$C$4+H36</f>
         <v>15</v>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="K36" s="8" t="n">
+      <c r="K36" s="9" t="n">
         <f aca="false">IF(I36&lt;=0,0,ROUNDUP(I36/J36,0))</f>
         <v>1</v>
       </c>
-      <c r="L36" s="18" t="n">
+      <c r="L36" s="19" t="n">
         <v>209.22</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="M36" s="15" t="n">
         <f aca="false">IF(L36="","",K36*L36)</f>
         <v>209.22</v>
       </c>
-      <c r="N36" s="15" t="s">
+      <c r="N36" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="O36" s="17" t="s">
+      <c r="O36" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="P36" s="16" t="s">
+      <c r="P36" s="17" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="8" t="n">
+    <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="C37" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D37" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="E37" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="F37" s="10" t="s">
+      <c r="F37" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="G37" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" s="12" t="n">
+      <c r="G37" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="I37" s="8" t="n">
+      <c r="I37" s="9" t="n">
         <f aca="false">G37*$C$4+H37</f>
         <v>1</v>
       </c>
-      <c r="J37" s="12" t="n">
+      <c r="J37" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="K37" s="8" t="n">
+      <c r="K37" s="9" t="n">
         <f aca="false">IF(I37&lt;=0,0,ROUNDUP(I37/J37,0))</f>
         <v>1</v>
       </c>
-      <c r="L37" s="13"/>
-      <c r="M37" s="14" t="str">
+      <c r="L37" s="14"/>
+      <c r="M37" s="15" t="str">
         <f aca="false">IF(L37="","",K37*L37)</f>
         <v/>
       </c>
-      <c r="N37" s="15"/>
-      <c r="O37" s="15"/>
-      <c r="P37" s="16" t="s">
+      <c r="N37" s="16"/>
+      <c r="O37" s="16"/>
+      <c r="P37" s="17" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L38" s="3" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="L38" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="M38" s="19" t="n">
+      <c r="M38" s="20" t="n">
         <f aca="false">SUM(M10:M37)</f>
         <v>459.81</v>
       </c>

</xml_diff>

<commit_message>
Dock: add six M3 mounting holes; BOM gets PCB price, USD rate cell and 1x19 socket note
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/dock/BOM.xlsx
+++ b/hardware/dock/BOM.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Dock BOM" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Dock BOM'!$A$9:$P$37</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Dock BOM'!$A$9:$P$34</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,10 +25,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>BOM</author>
+    <author>Claude</author>
+    <author>None</author>
   </authors>
   <commentList>
-    <comment ref="C5" authorId="0">
+    <comment ref="C5" authorId="1">
       <text>
         <r>
           <rPr>
@@ -40,12 +41,24 @@
         </r>
       </text>
     </comment>
+    <comment ref="C8" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">open.er-api.com USD→TRY on 2026-09-26: 48.92. Update before ordering.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="166">
   <si>
     <t xml:space="preserve">Dock-pad — Dock PCB bill of materials</t>
   </si>
@@ -74,7 +87,10 @@
     <t xml:space="preserve">Lines still missing a price</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue prices were seen on the listed shop on 2026-09-24 — verify before ordering. USD prices: convert to TL first.</t>
+    <t xml:space="preserve">Blue prices were seen on the listed shop on 2026-09-24 — verify before ordering. USD prices: multiply by the rate in C8.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USD → TL rate</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -134,13 +150,19 @@
     <t xml:space="preserve">Host + BLE module</t>
   </si>
   <si>
-    <t xml:space="preserve">Raspberry Pi Pico 2 WH</t>
+    <t xml:space="preserve">Raspberry Pi Pico 2 W</t>
   </si>
   <si>
     <t xml:space="preserve">Socketed, 2×20 headers</t>
   </si>
   <si>
-    <t xml:space="preserve">H version (headers pre-soldered). Remove the JST-SH debug connector and fit a 1×3 male header in the debug holes, pointing down</t>
+    <t xml:space="preserve">Robotistan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.robotistan.com/raspberry-pi-pico-2-w-header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solder male 1×20 headers + a 1×3 header on the debug holes (pointing down)</t>
   </si>
   <si>
     <t xml:space="preserve">A2, A3</t>
@@ -149,10 +171,13 @@
     <t xml:space="preserve">HID endpoint modules</t>
   </si>
   <si>
-    <t xml:space="preserve">Raspberry Pi Pico 2 H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H version (headers pre-soldered). JST debug connector can stay; SWD is via pogo probes on the bottom pads</t>
+    <t xml:space="preserve">Raspberry Pi Pico 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.robotistan.com/raspberry-pi-pico-2-header?language=tr&amp;h=7e0eb27a&amp;_sgm_campaign=fcs_c12e1a8d78000&amp;_sgm_source=12938%7Cproduct&amp;_sgm_action=search&amp;_sgm_term=pico&amp;_sgm_pinned=false</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solder male 1×20 headers (pointing down)</t>
   </si>
   <si>
     <t xml:space="preserve">ICs</t>
@@ -170,10 +195,10 @@
     <t xml:space="preserve">SOT-583-8 (hand-solder footprint)</t>
   </si>
   <si>
-    <t xml:space="preserve">LCSC (C3235557)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.lcsc.com/product-detail/C3235557.html</t>
+    <t xml:space="preserve">tme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.tme.eu/tr/tr/details/tps2116drlr/analog-coklayicilar-ve-anahtarlar/texas-instruments/</t>
   </si>
   <si>
     <t xml:space="preserve">Seen at LCSC for ~0.25 USD (2026-09-24). Tiny 0.5 mm pitch — spares recommended</t>
@@ -242,6 +267,9 @@
     <t xml:space="preserve">USB-C 16-pin SMD</t>
   </si>
   <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/usb-konnektorler-357/kls-electronic-l-kls1-5416-l1-01-r-1564461</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fine-pitch pads — spares for practice</t>
   </si>
   <si>
@@ -257,6 +285,12 @@
     <t xml:space="preserve">THT 1×6, 2.54 mm</t>
   </si>
   <si>
+    <t xml:space="preserve">Motorbit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.motorobit.com/6-pin-254mm-90c-pogo-pin-magnetic-connector-set-with-ear?srsltid=AU7gw4X13e_PdnJaSYcjqRrRIxg3XB_G7ziLdFPaJnamQ-Cs_lbV83Cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">GND | +5V | DET | RX | TX | GND</t>
   </si>
   <si>
@@ -272,6 +306,9 @@
     <t xml:space="preserve">THT</t>
   </si>
   <si>
+    <t xml:space="preserve">https://www.motorobit.com/1x40-erkek-header-40-pin-254mm-180-derece</t>
+  </si>
+  <si>
     <t xml:space="preserve">Can be cut from a 1×40 strip</t>
   </si>
   <si>
@@ -302,133 +339,190 @@
     <t xml:space="preserve">1 µF, ≥10 V, X7R</t>
   </si>
   <si>
+    <t xml:space="preserve">samsung CL21B105KBFNNNE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805 capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/smt-smd-ve-mlcc-kapasitorler-184/samsung-cl21b105kbfnnne-347740?catSequenceId=184</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1, C2, C10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 nF, ≥16 V, X7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">samsung CL21B104KBCNNNC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/smt-smd-ve-mlcc-kapasitorler-184/samsung-cl21b104kbcnnnc-14777?catSequenceId=184</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shield termination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3, R6, R13, R17, R18, R24, R29, R30, R31, R32, R36, R37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 kΩ 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805S8F1002T5E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805 resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f1002t5e-30240?catSequenceId=194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R25, R26, R27, R33, R34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 kΩ 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-071KL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/yageo-rc0805fr-071kl-460155?catSequenceId=194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R11, R12, R15, R16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.1 kΩ 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805S8F5101T5E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f5101t5e-358456?catSequenceId=194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB-C CC pull-downs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R9, R10, R14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">330 Ω 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805S8F3300T5E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f3300t5e-36831?catSequenceId=194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5, R23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.1 kΩ 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805S8F2612T5E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f2612t5e-505551?catSequenceId=194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sets the 1 A current limit (U3, U8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R7, R8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">56 kΩ 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805S8F5602T5E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f5602t5e-340670?catSequenceId=194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keyboard-port CC pull-ups</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R19, R21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 kΩ 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805S8F2202T5E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f2202t5e-335040?catSequenceId=194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VBUS sense divider (top)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R20, R22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33 kΩ 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805S8F3302T5E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f3302t5e-339608?catSequenceId=194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VBUS sense divider (bottom)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2, R28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 kΩ 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805S8F1003T5E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f1003t5e-30244?catSequenceId=194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">300 kΩ 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805S8F3003T5E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPS2116 PR1 divider (≈4.0 V switchover)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mechanical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Female socket 2.54 mm, 8.5 mm tall (cut from 1×40)</t>
+  </si>
+  <si>
     <t xml:space="preserve">generic</t>
   </si>
   <si>
-    <t xml:space="preserve">0805 capacitor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1, C2, C10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 nF, ≥16 V, X7R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shield termination</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3, R6, R13, R17, R18, R24, R29, R30, R31, R32, R36, R37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 kΩ 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0805 resistor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R25, R26, R27, R33, R34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 kΩ 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R11, R12, R15, R16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.1 kΩ 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB-C CC pull-downs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R9, R10, R14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">330 Ω 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5, R23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.1 kΩ 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sets the 1 A current limit (U3, U8)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R7, R8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">56 kΩ 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keyboard-port CC pull-ups</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R19, R21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22 kΩ 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VBUS sense divider (top)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R20, R22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">33 kΩ 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VBUS sense divider (bottom)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2, R28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 kΩ 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">300 kΩ 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TPS2116 PR1 divider (≈4.0 V switchover)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mechanical</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Female socket 1×20, 2.54 mm, 8.5 mm tall</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 per Pico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Female socket 1×3, 2.54 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">On the dock, under the host Pico 2 WH debug holes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Male pin header 1×20, 2.54 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not needed: H-version Picos come with headers pre-soldered</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Male pin header 1×3, 2.54 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaces the JST-SH debug connector on the host Pico 2 WH, pointing down into the 1×3 socket</t>
+    <t xml:space="preserve">motorbit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.motorobit.com/1x40-disi-header-40-pin-180-derece</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One 1×40 strip gives one 1×20 + one 1×19 (a pin is lost at the cut). Put the 1×19 on the pin 1–20 side, leaving pin 1 or 20 empty: GP0 and GP15 are unused on all three Picos</t>
   </si>
   <si>
     <t xml:space="preserve">Spring probe P50-B1</t>
@@ -440,10 +534,7 @@
     <t xml:space="preserve">0.68 mm barrel, 16.35 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">direnc.net</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.direnc.net/yayli-pogo-p50-b1-test-probu-13847</t>
+    <t xml:space="preserve">https://www.motorobit.com/yayli-pogo-p50-b1-test-probu-100-adet</t>
   </si>
   <si>
     <t xml:space="preserve">10 required + 5 optional (GND). Sold as 100-pack; price seen 2026-09-24 — verify</t>
@@ -458,7 +549,10 @@
     <t xml:space="preserve">JLCPCB / PCBWay</t>
   </si>
   <si>
-    <t xml:space="preserve">Sold per order of 5 (JLCPCB). Add shipping + import taxes separately</t>
+    <t xml:space="preserve">JLCPCB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.52 USD for 5 boards incl. e-post shipping to my address (JLCPCB quote 2026-09-26). Import taxes not included</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -468,17 +562,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00&quot; TL&quot;"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="0.00"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
@@ -499,6 +594,7 @@
     <font>
       <b val="true"/>
       <sz val="14"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -514,6 +610,7 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -535,11 +632,20 @@
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
@@ -629,12 +735,8 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -650,7 +752,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -659,6 +761,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -686,11 +792,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -698,19 +804,23 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -723,7 +833,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -735,6 +845,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -832,9 +950,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Sheets">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
@@ -842,10 +960,10 @@
         <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="4F81BD"/>
@@ -869,77 +987,19 @@
         <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="0000FF"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Sheets">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:ea typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:cs typeface="Calibri" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:cs typeface="Calibri" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -951,54 +1011,63 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
+                <a:lumMod val="110000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
+                <a:lumMod val="105000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
+                <a:lumMod val="105000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
           <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
+                <a:lumMod val="99000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
           <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -1016,46 +1085,34 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
+                <a:tint val="93000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
+                <a:tint val="98000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:shade val="63000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
           <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
@@ -1069,149 +1126,158 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P38"/>
-  <sheetFormatPr defaultColWidth="8.6171875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:P997"/>
+  <sheetFormatPr defaultColWidth="14.4296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="17" style="0" width="8.57"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="4" t="s">
+      <c r="C4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="6" t="n">
-        <f aca="false">SUM(M10:M37)</f>
-        <v>459.81</v>
-      </c>
-      <c r="E5" s="7" t="s">
+      <c r="C5" s="5" t="n">
+        <f aca="false">SUM(M10:M34)</f>
+        <v>3499.961</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="4" t="n">
-        <f aca="false">COUNT(L10:L37)</f>
-        <v>5</v>
-      </c>
-      <c r="E6" s="7" t="s">
+      <c r="C6" s="3" t="n">
+        <f aca="false">COUNT(L10:L34)</f>
+        <v>25</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="4" t="n">
-        <f aca="false">COUNTBLANK(L10:L37)</f>
-        <v>23</v>
-      </c>
-      <c r="E7" s="7" t="s">
+      <c r="C7" s="3" t="n">
+        <f aca="false">COUNTBLANK(L10:L34)</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>48.92</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M9" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="N9" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O9" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P9" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="n">
         <v>1</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G10" s="12" t="n">
         <v>1</v>
@@ -1230,35 +1296,41 @@
         <f aca="false">IF(I10&lt;=0,0,ROUNDUP(I10/J10,0))</f>
         <v>1</v>
       </c>
-      <c r="L10" s="14"/>
-      <c r="M10" s="15" t="str">
+      <c r="L10" s="14" t="n">
+        <v>559.61</v>
+      </c>
+      <c r="M10" s="15" t="n">
         <f aca="false">IF(L10="","",K10*L10)</f>
-        <v/>
-      </c>
-      <c r="N10" s="16"/>
-      <c r="O10" s="16"/>
-      <c r="P10" s="17" t="s">
-        <v>31</v>
+        <v>559.61</v>
+      </c>
+      <c r="N10" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="O10" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="P10" s="18" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="n">
         <v>2</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G11" s="12" t="n">
         <v>2</v>
@@ -1277,86 +1349,94 @@
         <f aca="false">IF(I11&lt;=0,0,ROUNDUP(I11/J11,0))</f>
         <v>2</v>
       </c>
-      <c r="L11" s="14"/>
-      <c r="M11" s="15" t="str">
+      <c r="L11" s="14" t="n">
+        <v>416.24</v>
+      </c>
+      <c r="M11" s="15" t="n">
         <f aca="false">IF(L11="","",K11*L11)</f>
-        <v/>
-      </c>
-      <c r="N11" s="16"/>
-      <c r="O11" s="16"/>
-      <c r="P11" s="17" t="s">
-        <v>35</v>
+        <v>832.48</v>
+      </c>
+      <c r="N11" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="O11" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="P11" s="18" t="s">
+        <v>39</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="n">
         <v>3</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G12" s="12" t="n">
         <v>1</v>
       </c>
       <c r="H12" s="13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I12" s="9" t="n">
         <f aca="false">G12*$C$4+H12</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J12" s="13" t="n">
         <v>1</v>
       </c>
       <c r="K12" s="9" t="n">
         <f aca="false">IF(I12&lt;=0,0,ROUNDUP(I12/J12,0))</f>
-        <v>3</v>
-      </c>
-      <c r="L12" s="14"/>
-      <c r="M12" s="15" t="str">
+        <v>5</v>
+      </c>
+      <c r="L12" s="14" t="n">
+        <v>34.31</v>
+      </c>
+      <c r="M12" s="15" t="n">
         <f aca="false">IF(L12="","",K12*L12)</f>
-        <v/>
+        <v>171.55</v>
       </c>
       <c r="N12" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="O12" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="P12" s="17" t="s">
-        <v>43</v>
+        <v>45</v>
+      </c>
+      <c r="O12" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="P12" s="18" t="s">
+        <v>47</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="n">
         <v>4</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G13" s="12" t="n">
         <v>1</v>
@@ -1375,7 +1455,7 @@
         <f aca="false">IF(I13&lt;=0,0,ROUNDUP(I13/J13,0))</f>
         <v>2</v>
       </c>
-      <c r="L13" s="19" t="n">
+      <c r="L13" s="20" t="n">
         <v>26.81</v>
       </c>
       <c r="M13" s="15" t="n">
@@ -1383,33 +1463,33 @@
         <v>53.62</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="O13" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="P13" s="17" t="s">
-        <v>50</v>
+        <v>52</v>
+      </c>
+      <c r="O13" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="P13" s="18" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="n">
         <v>5</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C14" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" s="11" t="s">
         <v>51</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>47</v>
       </c>
       <c r="G14" s="12" t="n">
         <v>1</v>
@@ -1428,7 +1508,7 @@
         <f aca="false">IF(I14&lt;=0,0,ROUNDUP(I14/J14,0))</f>
         <v>2</v>
       </c>
-      <c r="L14" s="19" t="n">
+      <c r="L14" s="20" t="n">
         <v>27.02</v>
       </c>
       <c r="M14" s="15" t="n">
@@ -1436,33 +1516,33 @@
         <v>54.04</v>
       </c>
       <c r="N14" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="O14" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="P14" s="17" t="s">
-        <v>55</v>
+        <v>52</v>
+      </c>
+      <c r="O14" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="P14" s="18" t="s">
+        <v>59</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="n">
         <v>6</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G15" s="12" t="n">
         <v>4</v>
@@ -1481,7 +1561,7 @@
         <f aca="false">IF(I15&lt;=0,0,ROUNDUP(I15/J15,0))</f>
         <v>6</v>
       </c>
-      <c r="L15" s="19" t="n">
+      <c r="L15" s="20" t="n">
         <v>11.88</v>
       </c>
       <c r="M15" s="15" t="n">
@@ -1489,33 +1569,33 @@
         <v>71.28</v>
       </c>
       <c r="N15" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="O15" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="P15" s="17" t="s">
-        <v>50</v>
+        <v>52</v>
+      </c>
+      <c r="O15" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="P15" s="18" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="n">
         <v>7</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G16" s="12" t="n">
         <v>3</v>
@@ -1534,35 +1614,41 @@
         <f aca="false">IF(I16&lt;=0,0,ROUNDUP(I16/J16,0))</f>
         <v>5</v>
       </c>
-      <c r="L16" s="14"/>
-      <c r="M16" s="15" t="str">
+      <c r="L16" s="14" t="n">
+        <v>4.164</v>
+      </c>
+      <c r="M16" s="15" t="n">
         <f aca="false">IF(L16="","",K16*L16)</f>
-        <v/>
-      </c>
-      <c r="N16" s="16"/>
-      <c r="O16" s="16"/>
-      <c r="P16" s="17" t="s">
-        <v>65</v>
+        <v>20.82</v>
+      </c>
+      <c r="N16" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O16" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="P16" s="18" t="s">
+        <v>70</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="n">
         <v>8</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="G17" s="12" t="n">
         <v>1</v>
@@ -1581,35 +1667,41 @@
         <f aca="false">IF(I17&lt;=0,0,ROUNDUP(I17/J17,0))</f>
         <v>1</v>
       </c>
-      <c r="L17" s="14"/>
-      <c r="M17" s="15" t="str">
+      <c r="L17" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="M17" s="15" t="n">
         <f aca="false">IF(L17="","",K17*L17)</f>
-        <v/>
-      </c>
-      <c r="N17" s="16"/>
-      <c r="O17" s="16"/>
-      <c r="P17" s="17" t="s">
-        <v>70</v>
+        <v>360</v>
+      </c>
+      <c r="N17" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="O17" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="P17" s="18" t="s">
+        <v>77</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="n">
         <v>9</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="G18" s="12" t="n">
         <v>3</v>
@@ -1622,41 +1714,47 @@
         <v>3</v>
       </c>
       <c r="J18" s="13" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K18" s="9" t="n">
         <f aca="false">IF(I18&lt;=0,0,ROUNDUP(I18/J18,0))</f>
-        <v>3</v>
-      </c>
-      <c r="L18" s="14"/>
-      <c r="M18" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L18" s="16" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M18" s="15" t="n">
         <f aca="false">IF(L18="","",K18*L18)</f>
-        <v/>
-      </c>
-      <c r="N18" s="16"/>
-      <c r="O18" s="16"/>
-      <c r="P18" s="17" t="s">
+        <v>3.6</v>
+      </c>
+      <c r="N18" s="16" t="s">
         <v>75</v>
       </c>
+      <c r="O18" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="P18" s="18" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="n">
         <v>10</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="G19" s="12" t="n">
         <v>4</v>
@@ -1675,7 +1773,7 @@
         <f aca="false">IF(I19&lt;=0,0,ROUNDUP(I19/J19,0))</f>
         <v>5</v>
       </c>
-      <c r="L19" s="19" t="n">
+      <c r="L19" s="14" t="n">
         <v>14.33</v>
       </c>
       <c r="M19" s="15" t="n">
@@ -1683,125 +1781,137 @@
         <v>71.65</v>
       </c>
       <c r="N19" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="O19" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="P19" s="17" t="s">
-        <v>82</v>
+        <v>52</v>
+      </c>
+      <c r="O19" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="P19" s="18" t="s">
+        <v>90</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="n">
         <v>11</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G20" s="12" t="n">
         <v>7</v>
       </c>
       <c r="H20" s="13" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="I20" s="9" t="n">
         <f aca="false">G20*$C$4+H20</f>
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="J20" s="13" t="n">
         <v>1</v>
       </c>
       <c r="K20" s="9" t="n">
         <f aca="false">IF(I20&lt;=0,0,ROUNDUP(I20/J20,0))</f>
-        <v>10</v>
-      </c>
-      <c r="L20" s="14"/>
-      <c r="M20" s="15" t="str">
+        <v>20</v>
+      </c>
+      <c r="L20" s="14" t="n">
+        <v>1.26923</v>
+      </c>
+      <c r="M20" s="15" t="n">
         <f aca="false">IF(L20="","",K20*L20)</f>
-        <v/>
-      </c>
-      <c r="N20" s="16"/>
-      <c r="O20" s="16"/>
-      <c r="P20" s="17"/>
+        <v>25.3846</v>
+      </c>
+      <c r="N20" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O20" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="P20" s="18"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="n">
         <v>12</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G21" s="12" t="n">
         <v>3</v>
       </c>
       <c r="H21" s="13" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I21" s="9" t="n">
         <f aca="false">G21*$C$4+H21</f>
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="J21" s="13" t="n">
         <v>1</v>
       </c>
       <c r="K21" s="9" t="n">
         <f aca="false">IF(I21&lt;=0,0,ROUNDUP(I21/J21,0))</f>
-        <v>5</v>
-      </c>
-      <c r="L21" s="14"/>
-      <c r="M21" s="15" t="str">
+        <v>20</v>
+      </c>
+      <c r="L21" s="14" t="n">
+        <v>0.5274</v>
+      </c>
+      <c r="M21" s="15" t="n">
         <f aca="false">IF(L21="","",K21*L21)</f>
-        <v/>
-      </c>
-      <c r="N21" s="16"/>
-      <c r="O21" s="16"/>
-      <c r="P21" s="17" t="s">
-        <v>89</v>
+        <v>10.548</v>
+      </c>
+      <c r="N21" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O21" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="P21" s="18" t="s">
+        <v>100</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="n">
         <v>13</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G22" s="12" t="n">
         <v>12</v>
@@ -1814,39 +1924,45 @@
         <v>15</v>
       </c>
       <c r="J22" s="13" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K22" s="9" t="n">
         <f aca="false">IF(I22&lt;=0,0,ROUNDUP(I22/J22,0))</f>
-        <v>15</v>
-      </c>
-      <c r="L22" s="14"/>
-      <c r="M22" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L22" s="14" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="M22" s="15" t="n">
         <f aca="false">IF(L22="","",K22*L22)</f>
-        <v/>
-      </c>
-      <c r="N22" s="16"/>
-      <c r="O22" s="16"/>
-      <c r="P22" s="17"/>
+        <v>10.68</v>
+      </c>
+      <c r="N22" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O22" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="P22" s="18"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="n">
         <v>14</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G23" s="12" t="n">
         <v>5</v>
@@ -1859,39 +1975,45 @@
         <v>7</v>
       </c>
       <c r="J23" s="13" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="K23" s="9" t="n">
         <f aca="false">IF(I23&lt;=0,0,ROUNDUP(I23/J23,0))</f>
-        <v>7</v>
-      </c>
-      <c r="L23" s="14"/>
-      <c r="M23" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L23" s="14" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="M23" s="15" t="n">
         <f aca="false">IF(L23="","",K23*L23)</f>
-        <v/>
-      </c>
-      <c r="N23" s="16"/>
-      <c r="O23" s="16"/>
-      <c r="P23" s="17"/>
+        <v>12.6</v>
+      </c>
+      <c r="N23" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O23" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="P23" s="18"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="n">
         <v>15</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>85</v>
+        <v>113</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G24" s="12" t="n">
         <v>4</v>
@@ -1904,41 +2026,47 @@
         <v>6</v>
       </c>
       <c r="J24" s="13" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K24" s="9" t="n">
         <f aca="false">IF(I24&lt;=0,0,ROUNDUP(I24/J24,0))</f>
-        <v>6</v>
-      </c>
-      <c r="L24" s="14"/>
-      <c r="M24" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L24" s="14" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="M24" s="15" t="n">
         <f aca="false">IF(L24="","",K24*L24)</f>
-        <v/>
-      </c>
-      <c r="N24" s="16"/>
-      <c r="O24" s="16"/>
-      <c r="P24" s="17" t="s">
-        <v>98</v>
+        <v>10.68</v>
+      </c>
+      <c r="N24" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O24" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="P24" s="18" t="s">
+        <v>115</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="n">
         <v>16</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G25" s="12" t="n">
         <v>3</v>
@@ -1951,39 +2079,45 @@
         <v>5</v>
       </c>
       <c r="J25" s="13" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K25" s="9" t="n">
         <f aca="false">IF(I25&lt;=0,0,ROUNDUP(I25/J25,0))</f>
-        <v>5</v>
-      </c>
-      <c r="L25" s="14"/>
-      <c r="M25" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L25" s="14" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="M25" s="15" t="n">
         <f aca="false">IF(L25="","",K25*L25)</f>
-        <v/>
-      </c>
-      <c r="N25" s="16"/>
-      <c r="O25" s="16"/>
-      <c r="P25" s="17"/>
+        <v>10.68</v>
+      </c>
+      <c r="N25" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O25" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="P25" s="18"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="n">
         <v>17</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>85</v>
+        <v>122</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G26" s="12" t="n">
         <v>2</v>
@@ -1996,41 +2130,47 @@
         <v>4</v>
       </c>
       <c r="J26" s="13" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K26" s="9" t="n">
         <f aca="false">IF(I26&lt;=0,0,ROUNDUP(I26/J26,0))</f>
-        <v>4</v>
-      </c>
-      <c r="L26" s="14"/>
-      <c r="M26" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L26" s="14" t="n">
+        <v>7.26</v>
+      </c>
+      <c r="M26" s="15" t="n">
         <f aca="false">IF(L26="","",K26*L26)</f>
-        <v/>
-      </c>
-      <c r="N26" s="16"/>
-      <c r="O26" s="16"/>
-      <c r="P26" s="17" t="s">
-        <v>103</v>
+        <v>7.26</v>
+      </c>
+      <c r="N26" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O26" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="P26" s="18" t="s">
+        <v>124</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="n">
         <v>18</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>104</v>
+        <v>125</v>
       </c>
       <c r="D27" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="F27" s="11" t="s">
         <v>105</v>
-      </c>
-      <c r="E27" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="F27" s="11" t="s">
-        <v>93</v>
       </c>
       <c r="G27" s="12" t="n">
         <v>2</v>
@@ -2043,41 +2183,47 @@
         <v>4</v>
       </c>
       <c r="J27" s="13" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K27" s="9" t="n">
         <f aca="false">IF(I27&lt;=0,0,ROUNDUP(I27/J27,0))</f>
-        <v>4</v>
-      </c>
-      <c r="L27" s="14"/>
-      <c r="M27" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L27" s="14" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="M27" s="15" t="n">
         <f aca="false">IF(L27="","",K27*L27)</f>
-        <v/>
-      </c>
-      <c r="N27" s="16"/>
-      <c r="O27" s="16"/>
-      <c r="P27" s="17" t="s">
-        <v>106</v>
+        <v>10.68</v>
+      </c>
+      <c r="N27" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O27" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="P27" s="18" t="s">
+        <v>129</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="n">
         <v>19</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>85</v>
+        <v>132</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G28" s="12" t="n">
         <v>2</v>
@@ -2090,41 +2236,47 @@
         <v>4</v>
       </c>
       <c r="J28" s="13" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K28" s="9" t="n">
         <f aca="false">IF(I28&lt;=0,0,ROUNDUP(I28/J28,0))</f>
-        <v>4</v>
-      </c>
-      <c r="L28" s="14"/>
-      <c r="M28" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L28" s="14" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="M28" s="15" t="n">
         <f aca="false">IF(L28="","",K28*L28)</f>
-        <v/>
-      </c>
-      <c r="N28" s="16"/>
-      <c r="O28" s="16"/>
-      <c r="P28" s="17" t="s">
-        <v>109</v>
+        <v>10.68</v>
+      </c>
+      <c r="N28" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O28" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="P28" s="18" t="s">
+        <v>134</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="n">
         <v>20</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>110</v>
+        <v>135</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>111</v>
+        <v>136</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>85</v>
+        <v>137</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G29" s="12" t="n">
         <v>2</v>
@@ -2137,41 +2289,47 @@
         <v>4</v>
       </c>
       <c r="J29" s="13" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K29" s="9" t="n">
         <f aca="false">IF(I29&lt;=0,0,ROUNDUP(I29/J29,0))</f>
-        <v>4</v>
-      </c>
-      <c r="L29" s="14"/>
-      <c r="M29" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L29" s="14" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="M29" s="15" t="n">
         <f aca="false">IF(L29="","",K29*L29)</f>
-        <v/>
-      </c>
-      <c r="N29" s="16"/>
-      <c r="O29" s="16"/>
-      <c r="P29" s="17" t="s">
-        <v>112</v>
+        <v>10.68</v>
+      </c>
+      <c r="N29" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O29" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="P29" s="18" t="s">
+        <v>139</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="n">
         <v>21</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>113</v>
+        <v>140</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>114</v>
+        <v>141</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>85</v>
+        <v>142</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G30" s="12" t="n">
         <v>2</v>
@@ -2184,39 +2342,45 @@
         <v>4</v>
       </c>
       <c r="J30" s="13" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K30" s="9" t="n">
         <f aca="false">IF(I30&lt;=0,0,ROUNDUP(I30/J30,0))</f>
-        <v>4</v>
-      </c>
-      <c r="L30" s="14"/>
-      <c r="M30" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L30" s="14" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="M30" s="15" t="n">
         <f aca="false">IF(L30="","",K30*L30)</f>
-        <v/>
-      </c>
-      <c r="N30" s="16"/>
-      <c r="O30" s="16"/>
-      <c r="P30" s="17"/>
+        <v>10.68</v>
+      </c>
+      <c r="N30" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O30" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="P30" s="18"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="n">
         <v>22</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>115</v>
+        <v>144</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>116</v>
+        <v>145</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>85</v>
+        <v>146</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G31" s="12" t="n">
         <v>1</v>
@@ -2229,335 +2393,1188 @@
         <v>3</v>
       </c>
       <c r="J31" s="13" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K31" s="9" t="n">
         <f aca="false">IF(I31&lt;=0,0,ROUNDUP(I31/J31,0))</f>
-        <v>3</v>
-      </c>
-      <c r="L31" s="14"/>
-      <c r="M31" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L31" s="14" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="M31" s="15" t="n">
         <f aca="false">IF(L31="","",K31*L31)</f>
-        <v/>
-      </c>
-      <c r="N31" s="16"/>
+        <v>10.68</v>
+      </c>
+      <c r="N31" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="O31" s="16"/>
-      <c r="P31" s="17" t="s">
-        <v>117</v>
+      <c r="P31" s="18" t="s">
+        <v>147</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="n">
         <v>23</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>85</v>
+        <v>151</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="G32" s="12" t="n">
         <v>6</v>
       </c>
       <c r="H32" s="13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I32" s="9" t="n">
         <f aca="false">G32*$C$4+H32</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J32" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K32" s="9" t="n">
         <f aca="false">IF(I32&lt;=0,0,ROUNDUP(I32/J32,0))</f>
-        <v>7</v>
-      </c>
-      <c r="L32" s="14"/>
-      <c r="M32" s="15" t="str">
+        <v>5</v>
+      </c>
+      <c r="L32" s="14" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="M32" s="15" t="n">
         <f aca="false">IF(L32="","",K32*L32)</f>
-        <v/>
-      </c>
-      <c r="N32" s="16"/>
-      <c r="O32" s="16"/>
-      <c r="P32" s="17" t="s">
-        <v>121</v>
+        <v>33</v>
+      </c>
+      <c r="N32" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="O32" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="P32" s="18" t="s">
+        <v>154</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>122</v>
+        <v>155</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>85</v>
+        <v>156</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>74</v>
+        <v>157</v>
       </c>
       <c r="G33" s="12" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="H33" s="13" t="n">
         <v>0</v>
       </c>
       <c r="I33" s="9" t="n">
         <f aca="false">G33*$C$4+H33</f>
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="J33" s="13" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K33" s="9" t="n">
         <f aca="false">IF(I33&lt;=0,0,ROUNDUP(I33/J33,0))</f>
         <v>1</v>
       </c>
-      <c r="L33" s="14"/>
-      <c r="M33" s="15" t="str">
+      <c r="L33" s="20" t="n">
+        <v>270</v>
+      </c>
+      <c r="M33" s="15" t="n">
         <f aca="false">IF(L33="","",K33*L33)</f>
-        <v/>
-      </c>
-      <c r="N33" s="16"/>
-      <c r="O33" s="16"/>
-      <c r="P33" s="17" t="s">
-        <v>123</v>
+        <v>270</v>
+      </c>
+      <c r="N33" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="O33" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="P33" s="18" t="s">
+        <v>159</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>118</v>
+        <v>28</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>160</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>124</v>
+        <v>161</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>85</v>
+        <v>162</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>74</v>
+        <v>149</v>
       </c>
       <c r="G34" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H34" s="13" t="n">
         <v>0</v>
       </c>
       <c r="I34" s="9" t="n">
         <f aca="false">G34*$C$4+H34</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34" s="13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K34" s="9" t="n">
         <f aca="false">IF(I34&lt;=0,0,ROUNDUP(I34/J34,0))</f>
-        <v>0</v>
-      </c>
-      <c r="L34" s="14"/>
-      <c r="M34" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L34" s="15" t="n">
+        <f aca="false">17.52*$C$8</f>
+        <v>857.0784</v>
+      </c>
+      <c r="M34" s="15" t="n">
         <f aca="false">IF(L34="","",K34*L34)</f>
-        <v/>
-      </c>
-      <c r="N34" s="16"/>
+        <v>857.0784</v>
+      </c>
+      <c r="N34" s="16" t="s">
+        <v>163</v>
+      </c>
       <c r="O34" s="16"/>
-      <c r="P34" s="17" t="s">
-        <v>125</v>
+      <c r="P34" s="18" t="s">
+        <v>164</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B35" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="C35" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="D35" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="E35" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="F35" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="G35" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H35" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="9" t="n">
-        <f aca="false">G35*$C$4+H35</f>
-        <v>1</v>
-      </c>
-      <c r="J35" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K35" s="9" t="n">
-        <f aca="false">IF(I35&lt;=0,0,ROUNDUP(I35/J35,0))</f>
-        <v>1</v>
-      </c>
-      <c r="L35" s="14"/>
-      <c r="M35" s="15" t="str">
-        <f aca="false">IF(L35="","",K35*L35)</f>
-        <v/>
-      </c>
-      <c r="N35" s="16"/>
-      <c r="O35" s="16"/>
-      <c r="P35" s="17" t="s">
-        <v>127</v>
+    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="L35" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="M35" s="21" t="n">
+        <f aca="false">SUM(M10:M34)</f>
+        <v>3499.961</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="C36" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="D36" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="E36" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="F36" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="G36" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="H36" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="9" t="n">
-        <f aca="false">G36*$C$4+H36</f>
-        <v>15</v>
-      </c>
-      <c r="J36" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="K36" s="9" t="n">
-        <f aca="false">IF(I36&lt;=0,0,ROUNDUP(I36/J36,0))</f>
-        <v>1</v>
-      </c>
-      <c r="L36" s="19" t="n">
-        <v>209.22</v>
-      </c>
-      <c r="M36" s="15" t="n">
-        <f aca="false">IF(L36="","",K36*L36)</f>
-        <v>209.22</v>
-      </c>
-      <c r="N36" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="O36" s="18" t="s">
-        <v>132</v>
-      </c>
-      <c r="P36" s="17" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="C37" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="D37" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="F37" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="G37" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" s="9" t="n">
-        <f aca="false">G37*$C$4+H37</f>
-        <v>1</v>
-      </c>
-      <c r="J37" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="K37" s="9" t="n">
-        <f aca="false">IF(I37&lt;=0,0,ROUNDUP(I37/J37,0))</f>
-        <v>1</v>
-      </c>
-      <c r="L37" s="14"/>
-      <c r="M37" s="15" t="str">
-        <f aca="false">IF(L37="","",K37*L37)</f>
-        <v/>
-      </c>
-      <c r="N37" s="16"/>
-      <c r="O37" s="16"/>
-      <c r="P37" s="17" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="L38" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="M38" s="20" t="n">
-        <f aca="false">SUM(M10:M37)</f>
-        <v>459.81</v>
-      </c>
-    </row>
+    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="114" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="115" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="116" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="117" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="118" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="119" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="120" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="121" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="122" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="123" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="124" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="125" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="126" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="127" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="128" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="129" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="130" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="131" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="132" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="133" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="134" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="149" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="150" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="151" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="152" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="153" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="154" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="155" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="158" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="159" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="160" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="169" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="170" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="172" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="175" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="176" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="178" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="179" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="180" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="181" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="182" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="183" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="184" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="185" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="186" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="187" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="188" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="189" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="190" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="191" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="192" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="193" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="194" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="196" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="197" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="199" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="200" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="201" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="202" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="203" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="204" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="205" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="206" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="207" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="208" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="209" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="210" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="211" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="212" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="213" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="214" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="215" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="216" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="217" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="218" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="219" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="220" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="221" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="222" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="223" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="224" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="225" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="226" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="227" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="228" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="229" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="230" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="231" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="232" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="233" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="234" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="235" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="236" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="237" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="238" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="239" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="240" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="241" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="242" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="243" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="244" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="245" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="246" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="247" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="248" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="249" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="250" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="251" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="252" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="253" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="254" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="255" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="256" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="257" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="258" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="259" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="260" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="261" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="262" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="263" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="264" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="265" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="266" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="267" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="268" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="269" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="270" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="271" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="272" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="273" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="274" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="275" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="276" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="277" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="278" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="279" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="280" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="281" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="282" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="283" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="284" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="285" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="286" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="287" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="288" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="289" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="290" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="291" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="292" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="293" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="294" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="295" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="296" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="297" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="298" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="299" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="300" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="301" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="302" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="303" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="304" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="305" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="306" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="307" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="308" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="309" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="310" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="311" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="312" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="313" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="314" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="315" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="316" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="317" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="318" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="319" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="320" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="321" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="322" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="323" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="324" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="325" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="326" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="327" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="328" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="329" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="330" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="331" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="332" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="333" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="334" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="335" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="336" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="337" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="338" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="339" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="340" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="341" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="342" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="343" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="344" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="345" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="346" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="347" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="348" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="349" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="350" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="351" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="352" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="353" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="354" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="355" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="356" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="357" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="358" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="359" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="360" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="361" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="362" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="363" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="364" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="365" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="366" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="367" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="368" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="369" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="370" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="371" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="372" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="373" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="374" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="375" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="376" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="377" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="378" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="379" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="380" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="381" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="382" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="383" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="384" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="385" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="386" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="387" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="388" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="389" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="390" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="391" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="392" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="393" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="394" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="395" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="396" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="397" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="398" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="399" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="400" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="401" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="402" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="403" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="404" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="405" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="406" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="407" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="408" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="409" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="410" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="411" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="412" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="413" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="414" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="415" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="416" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="417" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="418" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="419" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="420" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="421" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="422" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="423" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="424" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="425" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="426" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="427" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="428" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="429" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="430" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="431" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="432" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="433" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="434" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="435" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="436" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="437" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="438" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="439" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="440" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="441" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="442" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="443" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="444" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="445" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="446" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="447" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="448" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="449" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="450" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="451" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="452" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="453" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="454" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="455" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="456" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="457" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="458" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="459" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="460" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="461" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="462" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="463" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="464" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="465" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="466" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="467" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="468" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="469" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="470" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="471" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="472" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="473" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="474" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="475" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="476" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="477" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="478" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="479" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="480" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="481" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="482" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="483" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="484" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="485" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="486" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="487" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="488" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="489" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="490" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="491" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="492" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="493" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="494" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="495" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="496" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="497" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="498" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="499" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="500" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="501" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="502" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="503" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="504" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="505" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="506" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="507" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="508" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="509" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="510" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="511" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="512" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="513" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="514" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="515" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="516" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="517" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="518" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="519" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="520" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="521" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="522" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="523" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="524" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="525" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="526" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="527" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="528" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="529" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="530" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="531" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="532" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="533" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="534" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="535" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="536" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="537" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="538" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="539" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="540" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="541" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="542" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="543" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="544" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="545" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="546" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="547" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="548" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="549" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="550" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="551" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="552" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="553" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="554" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="555" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="556" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="557" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="558" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="559" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="560" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="561" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="562" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="563" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="564" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="565" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="566" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="567" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="568" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="569" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="570" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="571" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="572" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="573" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="574" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="575" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="576" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="577" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="578" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="579" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="580" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="581" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="582" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="583" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="584" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="585" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="586" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="587" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="588" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="589" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="590" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="591" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="592" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="593" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="594" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="595" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="596" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="597" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="598" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="599" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="600" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="601" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="602" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="603" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="604" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="605" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="606" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="607" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="608" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="609" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="610" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="611" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="612" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="613" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="614" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="615" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="616" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="617" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="618" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="619" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="620" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="621" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="622" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="623" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="624" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="625" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="626" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="627" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="628" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="629" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="630" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="631" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="632" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="633" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="634" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="635" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="636" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="637" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="638" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="639" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="640" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="641" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="642" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="643" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="644" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="645" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="646" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="647" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="648" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="649" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="650" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="651" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="652" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="653" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="654" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="655" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="656" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="657" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="658" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="659" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="660" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="661" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="662" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="663" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="664" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="665" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="666" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="667" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="668" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="669" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="670" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="671" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="672" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="673" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="674" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="675" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="676" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="677" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="678" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="679" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="680" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="681" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="682" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="683" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="684" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="685" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="686" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="687" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="688" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="689" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="690" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="691" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="692" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="693" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="694" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="695" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="696" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="697" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="698" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="699" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="700" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="701" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="702" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="703" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="704" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="705" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="706" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="707" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="708" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="709" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="710" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="711" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="712" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="713" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="714" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="715" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="716" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="717" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="718" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="719" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="720" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="721" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="722" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="723" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="724" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="725" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="726" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="727" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="728" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="729" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="730" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="731" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="732" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="733" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="734" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="735" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="736" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="737" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="738" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="739" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="740" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="741" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="742" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="743" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="744" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="745" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="746" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="747" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="748" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="749" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="750" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="751" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="752" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="753" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="754" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="755" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="756" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="757" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="758" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="759" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="760" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="761" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="762" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="763" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="764" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="765" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="766" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="767" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="768" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="769" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="770" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="771" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="772" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="773" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="774" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="775" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="776" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="777" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="778" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="779" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="780" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="781" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="782" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="783" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="784" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="785" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="786" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="787" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="788" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="789" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="790" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="791" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="792" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="793" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="794" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="795" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="796" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="797" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="798" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="799" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="800" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="801" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="802" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="803" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="804" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="805" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="806" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="807" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="808" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="809" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="810" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="811" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="812" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="813" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="814" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="815" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="816" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="817" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="818" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="819" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="820" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="821" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="822" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="823" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="824" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="825" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="826" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="827" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="828" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="829" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="830" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="831" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="832" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="833" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="834" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="835" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="836" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="837" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="838" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="839" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="840" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="841" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="842" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="843" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="844" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="845" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="846" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="847" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="848" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="849" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="850" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="851" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="852" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="853" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="854" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="855" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="856" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="857" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="858" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="859" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="860" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="861" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="862" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="863" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="864" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="865" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="866" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="867" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="868" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="869" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="870" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="871" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="872" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="873" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="874" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="875" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="876" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="877" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="878" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="879" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="880" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="881" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="882" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="883" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="884" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="885" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="886" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="887" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="888" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="889" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="890" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="891" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="892" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="893" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="894" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="895" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="896" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="897" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="898" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="899" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="900" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="901" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="902" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="903" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="904" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="905" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="906" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="907" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="908" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="909" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="910" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="911" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="912" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="913" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="914" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="915" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="916" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="917" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="918" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="919" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="920" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="921" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="922" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="923" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="924" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="925" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="926" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="927" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="928" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="929" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="930" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="931" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="932" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="933" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="934" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="935" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="936" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="937" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="938" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="939" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="940" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="941" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="942" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="943" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="944" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="945" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="946" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="947" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="948" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="949" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="950" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="951" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="952" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="953" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="954" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="955" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="956" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="957" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="958" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="959" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="960" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="961" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="962" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="963" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="964" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="965" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="966" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="967" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="968" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="969" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="970" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="971" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="972" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="973" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="974" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="975" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="976" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="977" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="978" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="979" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="980" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="981" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="982" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="983" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="984" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="985" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="986" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="987" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="988" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="989" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="990" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="991" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="992" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="993" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="994" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="995" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="996" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="997" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A9:P37"/>
+  <autoFilter ref="A9:P34"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L37" type="decimal">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L34" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="O12" r:id="rId2" display="https://www.lcsc.com/product-detail/C3235557.html"/>
-    <hyperlink ref="O13" r:id="rId3" display="https://ozdisan.com/integrated-circuits-ics/power-management-ics/power-switches/TPS2553DBVR"/>
-    <hyperlink ref="O14" r:id="rId4" display="https://ozdisan.com/integrated-circuits-ics/power-management-ics/power-switches/TPS2552DBVR"/>
-    <hyperlink ref="O15" r:id="rId5" display="https://ozdisan.com/power-semiconductors/diodes-diode-modules-and-rectifiers/tvs-diodes/TPD4E1U06DBVR"/>
-    <hyperlink ref="O19" r:id="rId6" display="https://www.ozdisan.com/passive-components/capacitors/aluminum-capacitors/EEE-FK1E101XP/622893"/>
-    <hyperlink ref="O36" r:id="rId7" display="https://www.direnc.net/yayli-pogo-p50-b1-test-probu-13847"/>
+    <hyperlink ref="O10" r:id="rId2" display="https://www.robotistan.com/raspberry-pi-pico-2-w-header"/>
+    <hyperlink ref="O11" r:id="rId3" display="https://www.robotistan.com/raspberry-pi-pico-2-header?language=tr&amp;h=7e0eb27a&amp;_sgm_campaign=fcs_c12e1a8d78000&amp;_sgm_source=12938%7Cproduct&amp;_sgm_action=search&amp;_sgm_term=pico&amp;_sgm_pinned=false"/>
+    <hyperlink ref="O12" r:id="rId4" display="https://www.tme.eu/tr/tr/details/tps2116drlr/analog-coklayicilar-ve-anahtarlar/texas-instruments/"/>
+    <hyperlink ref="O13" r:id="rId5" display="https://ozdisan.com/integrated-circuits-ics/power-management-ics/power-switches/TPS2553DBVR"/>
+    <hyperlink ref="O14" r:id="rId6" display="https://ozdisan.com/integrated-circuits-ics/power-management-ics/power-switches/TPS2552DBVR"/>
+    <hyperlink ref="O15" r:id="rId7" display="https://ozdisan.com/power-semiconductors/diodes-diode-modules-and-rectifiers/tvs-diodes/TPD4E1U06DBVR"/>
+    <hyperlink ref="O16" r:id="rId8" display="https://www.ozdisan.com/p/usb-konnektorler-357/kls-electronic-l-kls1-5416-l1-01-r-1564461"/>
+    <hyperlink ref="O17" r:id="rId9" display="https://www.motorobit.com/6-pin-254mm-90c-pogo-pin-magnetic-connector-set-with-ear?srsltid=AU7gw4X13e_PdnJaSYcjqRrRIxg3XB_G7ziLdFPaJnamQ-Cs_lbV83Cm"/>
+    <hyperlink ref="O18" r:id="rId10" display="https://www.motorobit.com/1x40-erkek-header-40-pin-254mm-180-derece"/>
+    <hyperlink ref="O19" r:id="rId11" display="https://www.ozdisan.com/passive-components/capacitors/aluminum-capacitors/EEE-FK1E101XP/622893"/>
+    <hyperlink ref="O20" r:id="rId12" display="https://www.ozdisan.com/p/smt-smd-ve-mlcc-kapasitorler-184/samsung-cl21b105kbfnnne-347740?catSequenceId=184"/>
+    <hyperlink ref="O21" r:id="rId13" display="https://www.ozdisan.com/p/smt-smd-ve-mlcc-kapasitorler-184/samsung-cl21b104kbcnnnc-14777?catSequenceId=184"/>
+    <hyperlink ref="O22" r:id="rId14" display="https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f1002t5e-30240?catSequenceId=194"/>
+    <hyperlink ref="O23" r:id="rId15" display="https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/yageo-rc0805fr-071kl-460155?catSequenceId=194"/>
+    <hyperlink ref="O24" r:id="rId16" display="https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f5101t5e-358456?catSequenceId=194"/>
+    <hyperlink ref="O25" r:id="rId17" display="https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f3300t5e-36831?catSequenceId=194"/>
+    <hyperlink ref="O26" r:id="rId18" display="https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f2612t5e-505551?catSequenceId=194"/>
+    <hyperlink ref="O27" r:id="rId19" display="https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f5602t5e-340670?catSequenceId=194"/>
+    <hyperlink ref="O28" r:id="rId20" display="https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f2202t5e-335040?catSequenceId=194"/>
+    <hyperlink ref="O29" r:id="rId21" display="https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f3302t5e-339608?catSequenceId=194"/>
+    <hyperlink ref="O30" r:id="rId22" display="https://www.ozdisan.com/p/smt-smd-ve-cip-direncler-194/royalohm-0805s8f1003t5e-30244?catSequenceId=194"/>
+    <hyperlink ref="O32" r:id="rId23" display="https://www.motorobit.com/1x40-disi-header-40-pin-180-derece"/>
+    <hyperlink ref="O33" r:id="rId24" display="https://www.motorobit.com/yayli-pogo-p50-b1-test-probu-100-adet"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2566,7 +3583,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId8"/>
-  <legacyDrawing r:id="rId9"/>
+  <drawing r:id="rId25"/>
+  <legacyDrawing r:id="rId26"/>
 </worksheet>
 </file>
</xml_diff>